<commit_message>
docs : update formular
</commit_message>
<xml_diff>
--- a/sprint_1/1_business_analysis/deliverables/AC_completed.xlsx
+++ b/sprint_1/1_business_analysis/deliverables/AC_completed.xlsx
@@ -340,19 +340,19 @@
     <t>Số liệu/xu hướng sử dụng điện tại [khu vực] trong [số] [ngày/tuần/tháng/năm] qua</t>
   </si>
   <si>
-    <t xml:space="preserve">Xu hướng sử dụng điện = So sánh lượng điện tiêu thụ theo ngày/tuần/tháng/năm; tốc độ tăng trưởng (%) = ((Kỳ hiện tại − Kỳ trước) / Kỳ trước) / 100. </t>
+    <t xml:space="preserve"> So sánh lượng điện tiêu thụ theo ngày/tuần/tháng/năm; tốc độ tăng trưởng (%) = ((Kỳ hiện tại − Kỳ trước) / Kỳ trước) / 100. </t>
   </si>
   <si>
     <t>Top [số] khu vực tiêu thụ điện [nhiều/ít] nhất</t>
   </si>
   <si>
-    <t>Top khu vực tiêu thụ điện = Sắp xếp tổng kWh tiêu thụ theo khu vực giảm dần/tăng dần trong khoảng thời gian xác định.</t>
+    <t xml:space="preserve"> Sắp xếp tổng kWh tiêu thụ theo khu vực giảm dần/tăng dần trong khoảng thời gian xác định.</t>
   </si>
   <si>
     <t>Tỉ lệ khả năng lưu trữ của mạng lưới điện hiện tại so với tổng lượng điện tiêu thụ</t>
   </si>
   <si>
-    <t xml:space="preserve">Tỉ lệ khả năng lưu trữ điện (%) = (Dung lượng lưu trữ của lưới điện hoặc hệ pin lưu trữ / Tổng điện năng tiêu thụ toàn thành phố) / 100. </t>
+    <t xml:space="preserve"> Dung lượng lưu trữ của lưới điện hoặc hệ pin lưu trữ / Tổng điện năng tiêu thụ toàn thành phố / 100. </t>
   </si>
   <si>
     <t>Danh sách các nguồn cấp điện bị quá tải</t>
@@ -364,19 +364,19 @@
     <t>Danh sách các hệ thống cấp nước bị hỏng</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh sách hệ thống cấp nước bị hỏng = Lọc các thiết bị/cảm biến/trạm cấp nước có trạng thái lỗi, mất kết nối hoặc không hoạt động. </t>
+    <t xml:space="preserve">Lọc các thiết bị/cảm biến/trạm cấp nước có trạng thái lỗi, mất kết nối hoặc không hoạt động. </t>
   </si>
   <si>
     <t>Số lượng đèn tín hiệu giao thông thông minh hiện tại, lọc theo trạng thái (hoạt động bình thường/hư hỏng)</t>
   </si>
   <si>
-    <t xml:space="preserve">Công thức tỷ lệ (%) = (Số đèn thông minh  có trạng thái được hỏi / Tổng số đèn tín hiệu) / 100. </t>
+    <t xml:space="preserve">Số đèn thông minh  có trạng thái được hỏi / Tổng số đèn tín hiệu / 100. </t>
   </si>
   <si>
     <t>Danh sách các đèn báo hiệu giao thông thông minh gặp vấn đề, bị hỏng.</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh sách đèn tín hiệu giao thông gặp sự cố = Lọc các đèn có trạng thái fault/offline/bảo trì trong hệ thống ITS. </t>
+    <t xml:space="preserve">Lọc các đèn có trạng thái fault/offline/bảo trì trong hệ thống ITS. </t>
   </si>
   <si>
     <t>Các tuyến đường đang ùn tắc hiện tại</t>
@@ -391,7 +391,7 @@
     <t>G</t>
   </si>
   <si>
-    <t xml:space="preserve">Danh sách camera gặp sự cố = Lọc camera có trạng thái offline, mất tín hiệu hoặc lỗi phần cứng/phần mềm. </t>
+    <t xml:space="preserve">Lọc camera có trạng thái offline, mất tín hiệu hoặc lỗi phần cứng/phần mềm. </t>
   </si>
   <si>
     <t>PHẦN 2: CÂU HỎI BỔ SUNG THÊM KHÔNG MAPPING VỚI ISO 37122 INDICATOR</t>
@@ -403,7 +403,7 @@
     <t>Lọc theo trạng thái / khu vực</t>
   </si>
   <si>
-    <t>Thiết bị ra/vào tòa nhà không hoạt động = Lọc thiết bị access control có trạng thái offline/lỗi/bảo trì theo khu vực.</t>
+    <t xml:space="preserve"> Lọc thiết bị access control có trạng thái offline/lỗi/bảo trì theo khu vực.</t>
   </si>
   <si>
     <t>Danh sách các thang máy đang trong trạng thái không hoạt động/hư hỏng/bảo trì</t>
@@ -415,31 +415,31 @@
     <t>Danh sách các hệ thống báo cháy đang trong trạng thái không hoạt động/hư hỏng/bảo trì</t>
   </si>
   <si>
-    <t xml:space="preserve">Hệ thống báo cháy không hoạt động = Lọc các cảm biến/tủ báo cháy có trạng thái lỗi, mất kết nối hoặc bảo trì. </t>
+    <t xml:space="preserve"> Lọc các cảm biến/tủ báo cháy có trạng thái lỗi, mất kết nối hoặc bảo trì. </t>
   </si>
   <si>
     <t>Danh sách các khu vực tiêu thụ nhiều điện năng nhất</t>
   </si>
   <si>
-    <t>Khu vực tiêu thụ điện năng nhiều nhất = Tổng hợp kWh tiêu thụ theo khu vực và sắp xếp giảm dần</t>
+    <t>Tổng hợp kWh tiêu thụ theo khu vực và sắp xếp giảm dần</t>
   </si>
   <si>
     <t xml:space="preserve">Danh sách các khu vực tiêu thụ nhiều  nước sinh hoạt  nhất </t>
   </si>
   <si>
-    <t xml:space="preserve">Khu vực tiêu thụ nước sinh hoạt nhiều nhất = Tổng hợp m3 nước tiêu thụ theo khu vực và sắp xếp giảm dần. </t>
+    <t xml:space="preserve"> Tổng hợp m3 nước tiêu thụ theo khu vực và sắp xếp giảm dần. </t>
   </si>
   <si>
     <t xml:space="preserve">Danh sách các khu vực đang có đường thi công , sửa chữa giao thông </t>
   </si>
   <si>
-    <t>Khu vực có đường thi công/sửa chữa = Lọc các tuyến đường có trạng thái công trình đang hoạt động trong hệ thống quản lý hạ tầng</t>
+    <t>Lọc các tuyến đường có trạng thái công trình đang hoạt động trong hệ thống quản lý hạ tầng</t>
   </si>
   <si>
     <t xml:space="preserve">Danh sách các khu vực đang đang thi công cơ sở hạ tầng (nhà ở ,  bến xe , ... )  </t>
   </si>
   <si>
-    <t>Khu vực đang thi công cơ sở hạ tầng = Lọc các dự án có trạng thái đang thi công theo khu vực trên hệ thống quản lý dự án/GIS đô thị</t>
+    <t>Lọc các dự án có trạng thái đang thi công theo khu vực trên hệ thống quản lý dự án/GIS đô thị</t>
   </si>
   <si>
     <t xml:space="preserve">Danh sách các khu vực có cây xanh bị thiệt hại </t>

</xml_diff>